<commit_message>
update common import export
</commit_message>
<xml_diff>
--- a/src/main/resources/i18n/common.xlsx
+++ b/src/main/resources/i18n/common.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Intellj\Micro\CoreCommon\src\main\resources\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A04C7ED4-44F7-46C3-B608-1BCF3B9D117D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA42BB32-0E34-441D-B6DC-E4A3256EEFDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E50E03D4-4F8A-4BB7-9FDA-052AF5257747}"/>
+    <workbookView xWindow="33000" yWindow="2250" windowWidth="21600" windowHeight="11460" xr2:uid="{E50E03D4-4F8A-4BB7-9FDA-052AF5257747}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>key</t>
   </si>
@@ -114,6 +114,18 @@
   </si>
   <si>
     <t>言語コードはサポートされていません</t>
+  </si>
+  <si>
+    <t>I18N_IMPORT_ERROR</t>
+  </si>
+  <si>
+    <t>Failed to import i18n file: {0}</t>
+  </si>
+  <si>
+    <t>Lỗi import file i18n: {0}</t>
+  </si>
+  <si>
+    <t>i18nファイルのインポートに失敗しました: {0}</t>
   </si>
 </sst>
 </file>
@@ -485,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CA4F4B4-AF50-4496-B9AC-762B42711D9F}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.375" bestFit="1" customWidth="1"/>
@@ -592,6 +604,20 @@
         <v>25</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
update department with role corresponding
</commit_message>
<xml_diff>
--- a/src/main/resources/i18n/common.xlsx
+++ b/src/main/resources/i18n/common.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Intellj\Testing\Common\src\main\resources\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5383B5DF-F04A-48FC-9751-0AA398493223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32F4A46-1BB1-4FE9-B54C-8D3857275608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6495" yWindow="1710" windowWidth="21600" windowHeight="11460" xr2:uid="{E50E03D4-4F8A-4BB7-9FDA-052AF5257747}"/>
+    <workbookView xWindow="9630" yWindow="4830" windowWidth="20835" windowHeight="9420" xr2:uid="{E50E03D4-4F8A-4BB7-9FDA-052AF5257747}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
   <si>
     <t>key</t>
   </si>
@@ -189,6 +189,18 @@
   </si>
   <si>
     <t>is_error</t>
+  </si>
+  <si>
+    <t>NOT_FOUND_COUNTRY</t>
+  </si>
+  <si>
+    <t>Không tìm thấy quốc gia</t>
+  </si>
+  <si>
+    <t>Country not found</t>
+  </si>
+  <si>
+    <t>国が見つかりません</t>
   </si>
 </sst>
 </file>
@@ -563,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CA4F4B4-AF50-4496-B9AC-762B42711D9F}">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.375" bestFit="1" customWidth="1"/>
@@ -789,6 +801,26 @@
       <c r="D13" t="s">
         <v>44</v>
       </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>